<commit_message>
ciclo 2026-06: 4b_reclamos completo, tests planilla/efectivo, datos e inputs junio
- 4b_reclamos: módulo nuevo completo (main.py, resolucion.py, docs HTML, tests, backup)
- 2_planilla: config y main actualizados + test_publicar_shared.py
- 3_boletas: correcciones.py + DATA_boletas actualizado
- 4_pagos/efectivo: README, mesa_1/5, tests integración/unitarios, trazabilidad 2026-06
- 5_cobranza: inputs actualizados (planilla, pagos_yape, pagos_efectivo) + backup 13-jun
- docs: metodologia v3.0, skill_tracker, decisiones 4b_reclamos, reporte aprendizaje 13-jun
- shared: blancos_acumulados y planilla_2026-06 actualizados

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_pagos/efectivo/inputs/mesa_1.xlsx
+++ b/4_pagos/efectivo/inputs/mesa_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilde\PycharmProjects\jass_system\4_pagos\efectivo\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC6018A3-E7B8-49EC-B0E3-5F6E83FF4C42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CE0D300-18C6-4674-886D-D3804FF3C8ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28905" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="registro_1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="56">
   <si>
     <t>¿Quién cobró?</t>
   </si>
@@ -195,6 +195,15 @@
   </si>
   <si>
     <t>pago parcial</t>
+  </si>
+  <si>
+    <t>reclamo_mes_actual</t>
+  </si>
+  <si>
+    <t>reclamo_mes_anterior</t>
+  </si>
+  <si>
+    <t>reclamo_convenio</t>
   </si>
 </sst>
 </file>
@@ -654,7 +663,7 @@
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="20.453125" customWidth="1"/>
+    <col min="9" max="9" width="35.36328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -787,7 +796,7 @@
         <v>46178</v>
       </c>
       <c r="I5" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
@@ -816,7 +825,7 @@
         <v>46178</v>
       </c>
       <c r="I6" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
@@ -874,7 +883,7 @@
         <v>46178</v>
       </c>
       <c r="I8" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
@@ -1266,9 +1275,6 @@
       </c>
       <c r="H22" s="8">
         <v>46178</v>
-      </c>
-      <c r="I22" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
ciclo 2026-06: 6_corte refactorizado · shared/repo pattern · 4b_reclamos completo
- 6_corte: reemplaza main.py monolítico por 3 scripts (generar_lista, aplicar_penalidad, seguimiento) + config + README + 8 contratos HTML
- 6b_override: eliminado (absorbido por 6_corte)
- 4b_reclamos: agrega aplicar_correcciones.py, dedupe_trazabilidad.py, validacion_resolucion_correcciones.py · actualiza main y resolucion
- shared: data_boletas_repo.py (único writer) · utils_lote.py · README · audit log · docs
- 5_cobranza: main + tests actualizados para junio 2026
- 4_pagos: efectivo/main y yape/validacion actualizados · mesas 1-6 actualizadas
- Data: planilla, pagos_efectivo, DATA_boletas, trazabilidades junio 2026
- docs: skill_tracker + metodologia v3.8 · reporte aprendizaje 20260616
- .gitignore: agrega exclusiones backup/ y tmp_*.py

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_pagos/efectivo/inputs/mesa_1.xlsx
+++ b/4_pagos/efectivo/inputs/mesa_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilde\PycharmProjects\jass_system\4_pagos\efectivo\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CE0D300-18C6-4674-886D-D3804FF3C8ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50537B49-E0D8-49B7-A719-3151832356AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25950" yWindow="615" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="registro_1" sheetId="1" r:id="rId1"/>
@@ -194,9 +194,6 @@
     <t>pago mixto</t>
   </si>
   <si>
-    <t>pago parcial</t>
-  </si>
-  <si>
     <t>reclamo_mes_actual</t>
   </si>
   <si>
@@ -204,6 +201,9 @@
   </si>
   <si>
     <t>reclamo_convenio</t>
+  </si>
+  <si>
+    <t>compromiso</t>
   </si>
 </sst>
 </file>
@@ -796,7 +796,7 @@
         <v>46178</v>
       </c>
       <c r="I5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
@@ -825,7 +825,7 @@
         <v>46178</v>
       </c>
       <c r="I6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
@@ -854,7 +854,7 @@
         <v>46178</v>
       </c>
       <c r="I7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
@@ -883,7 +883,7 @@
         <v>46178</v>
       </c>
       <c r="I8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">

</xml_diff>